<commit_message>
normalised with ratio method
</commit_message>
<xml_diff>
--- a/src/data/calibration_data_blue.xlsx
+++ b/src/data/calibration_data_blue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matthew Tan\Documents\ECSE211\ECSE211_W26_Final_Project\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{84840E61-0067-4ED7-ABA6-57C536990C9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5337C0F-740F-4FC6-9CC3-2862ACC68FC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CC244277-A238-44C5-9F20-A74BC72E50A2}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>R</t>
   </si>
@@ -44,10 +44,16 @@
     <t>B</t>
   </si>
   <si>
-    <t>avg</t>
+    <t>vector avg</t>
   </si>
   <si>
-    <t>std dev</t>
+    <t>vector std dev</t>
+  </si>
+  <si>
+    <t>ratio avg</t>
+  </si>
+  <si>
+    <t>ratio std dev</t>
   </si>
 </sst>
 </file>
@@ -908,10 +914,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8088C93-D36D-44C3-A782-AA40B20A4263}">
-  <dimension ref="A1:M90"/>
+  <dimension ref="A1:Q90"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="14" max="14" width="11.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -922,7 +931,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>38</v>
       </c>
@@ -944,23 +953,35 @@
         <f t="shared" si="0"/>
         <v>6.3848411513310332E-3</v>
       </c>
-      <c r="J2" t="s">
+      <c r="I2">
+        <f>A2/($A2+$B2+$C2)</f>
+        <v>0.17840375586854459</v>
+      </c>
+      <c r="J2">
+        <f t="shared" ref="J2:K2" si="1">B2/($A2+$B2+$C2)</f>
+        <v>0.23943661971830985</v>
+      </c>
+      <c r="K2">
+        <f t="shared" si="1"/>
+        <v>0.5821596244131455</v>
+      </c>
+      <c r="N2" t="s">
         <v>3</v>
       </c>
-      <c r="K2">
+      <c r="O2">
         <f>AVERAGE(E2:E90)</f>
         <v>1.8933099036467552E-3</v>
       </c>
-      <c r="L2">
-        <f t="shared" ref="L2:M2" si="1">AVERAGE(F2:F90)</f>
+      <c r="P2">
+        <f>AVERAGE(F2:F90)</f>
         <v>2.5693768305754387E-3</v>
       </c>
-      <c r="M2">
-        <f t="shared" si="1"/>
+      <c r="Q2">
+        <f>AVERAGE(G2:G90)</f>
         <v>5.5279132291140756E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>43</v>
       </c>
@@ -982,23 +1003,35 @@
         <f t="shared" ref="G3:G66" si="4">C3/($A3^2 + $B3^2 + $C3^2)</f>
         <v>6.1652909405890141E-3</v>
       </c>
-      <c r="J3" t="s">
+      <c r="I3">
+        <f t="shared" ref="I3:I66" si="5">A3/($A3+$B3+$C3)</f>
+        <v>0.19545454545454546</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J66" si="6">B3/($A3+$B3+$C3)</f>
+        <v>0.25454545454545452</v>
+      </c>
+      <c r="K3">
+        <f t="shared" ref="K3:K66" si="7">C3/($A3+$B3+$C3)</f>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="N3" t="s">
         <v>4</v>
       </c>
-      <c r="K3">
+      <c r="O3">
         <f>_xlfn.STDEV.P(E2:E90)</f>
         <v>2.5989942313835439E-4</v>
       </c>
-      <c r="L3">
-        <f t="shared" ref="L3:M3" si="5">_xlfn.STDEV.P(F2:F90)</f>
+      <c r="P3">
+        <f>_xlfn.STDEV.P(F2:F90)</f>
         <v>3.1193394626502388E-4</v>
       </c>
-      <c r="M3">
-        <f t="shared" si="5"/>
+      <c r="Q3">
+        <f>_xlfn.STDEV.P(G2:G90)</f>
         <v>7.8037261431361299E-4</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>41</v>
       </c>
@@ -1020,8 +1053,20 @@
         <f t="shared" si="4"/>
         <v>6.1925790569006649E-3</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I4">
+        <f t="shared" si="5"/>
+        <v>0.18721461187214611</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="6"/>
+        <v>0.25570776255707761</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="7"/>
+        <v>0.55707762557077622</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>40</v>
       </c>
@@ -1043,8 +1088,35 @@
         <f t="shared" si="4"/>
         <v>6.3438359061112285E-3</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I5">
+        <f t="shared" si="5"/>
+        <v>0.18691588785046728</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="6"/>
+        <v>0.25233644859813081</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="7"/>
+        <v>0.56074766355140182</v>
+      </c>
+      <c r="N5" t="s">
+        <v>5</v>
+      </c>
+      <c r="O5">
+        <f>AVERAGE(I2:I90)</f>
+        <v>0.18948403717301232</v>
+      </c>
+      <c r="P5">
+        <f t="shared" ref="P5:Q5" si="8">AVERAGE(J2:J90)</f>
+        <v>0.25771120806584513</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" si="8"/>
+        <v>0.55280475476114233</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>42</v>
       </c>
@@ -1066,8 +1138,35 @@
         <f t="shared" si="4"/>
         <v>6.1315776247675528E-3</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I6">
+        <f t="shared" si="5"/>
+        <v>0.19004524886877827</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="6"/>
+        <v>0.25791855203619912</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="7"/>
+        <v>0.55203619909502266</v>
+      </c>
+      <c r="N6" t="s">
+        <v>6</v>
+      </c>
+      <c r="O6">
+        <f>_xlfn.STDEV.P(I2:I90)</f>
+        <v>3.7983423784507873E-3</v>
+      </c>
+      <c r="P6">
+        <f t="shared" ref="P6:Q6" si="9">_xlfn.STDEV.P(J2:J90)</f>
+        <v>4.9166661361926258E-3</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="9"/>
+        <v>6.6441351887760848E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>40</v>
       </c>
@@ -1089,8 +1188,20 @@
         <f t="shared" si="4"/>
         <v>6.4081852450188475E-3</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I7">
+        <f t="shared" si="5"/>
+        <v>0.18867924528301888</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="6"/>
+        <v>0.25</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="7"/>
+        <v>0.56132075471698117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>41</v>
       </c>
@@ -1112,8 +1223,20 @@
         <f t="shared" si="4"/>
         <v>6.1925790569006649E-3</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I8">
+        <f t="shared" si="5"/>
+        <v>0.18721461187214611</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="6"/>
+        <v>0.25570776255707761</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="7"/>
+        <v>0.55707762557077622</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>40</v>
       </c>
@@ -1135,8 +1258,20 @@
         <f t="shared" si="4"/>
         <v>6.4081852450188475E-3</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I9">
+        <f t="shared" si="5"/>
+        <v>0.18867924528301888</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="6"/>
+        <v>0.25</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="7"/>
+        <v>0.56132075471698117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>42</v>
       </c>
@@ -1158,8 +1293,20 @@
         <f t="shared" si="4"/>
         <v>6.1921088992375004E-3</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I10">
+        <f t="shared" si="5"/>
+        <v>0.19178082191780821</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="6"/>
+        <v>0.25570776255707761</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="7"/>
+        <v>0.55251141552511418</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>39</v>
       </c>
@@ -1181,8 +1328,20 @@
         <f t="shared" si="4"/>
         <v>6.3781561330451741E-3</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I11">
+        <f t="shared" si="5"/>
+        <v>0.18309859154929578</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="6"/>
+        <v>0.24882629107981222</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="7"/>
+        <v>0.568075117370892</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>43</v>
       </c>
@@ -1204,8 +1363,20 @@
         <f t="shared" si="4"/>
         <v>6.1903533660046424E-3</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I12">
+        <f t="shared" si="5"/>
+        <v>0.19634703196347031</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="6"/>
+        <v>0.25570776255707761</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="7"/>
+        <v>0.54794520547945202</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>41</v>
       </c>
@@ -1227,8 +1398,20 @@
         <f t="shared" si="4"/>
         <v>6.2807495027739973E-3</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I13">
+        <f t="shared" si="5"/>
+        <v>0.18981481481481483</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="6"/>
+        <v>0.25462962962962965</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="7"/>
+        <v>0.55555555555555558</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>43</v>
       </c>
@@ -1250,8 +1433,20 @@
         <f t="shared" si="4"/>
         <v>6.1054949454509054E-3</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I14">
+        <f t="shared" si="5"/>
+        <v>0.19369369369369369</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="6"/>
+        <v>0.25675675675675674</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="7"/>
+        <v>0.5495495495495496</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>41</v>
       </c>
@@ -1273,8 +1468,20 @@
         <f t="shared" si="4"/>
         <v>6.3167868610833292E-3</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I15">
+        <f t="shared" si="5"/>
+        <v>0.19069767441860466</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="6"/>
+        <v>0.25116279069767444</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="7"/>
+        <v>0.55813953488372092</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>43</v>
       </c>
@@ -1296,8 +1503,20 @@
         <f t="shared" si="4"/>
         <v>6.1299964537210603E-3</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I16">
+        <f t="shared" si="5"/>
+        <v>0.19457013574660634</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="6"/>
+        <v>0.25791855203619912</v>
+      </c>
+      <c r="K16">
+        <f t="shared" si="7"/>
+        <v>0.54751131221719462</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>43</v>
       </c>
@@ -1319,8 +1538,20 @@
         <f t="shared" si="4"/>
         <v>6.2516417126346202E-3</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I17">
+        <f t="shared" si="5"/>
+        <v>0.19815668202764977</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="6"/>
+        <v>0.25345622119815669</v>
+      </c>
+      <c r="K17">
+        <f t="shared" si="7"/>
+        <v>0.54838709677419351</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>43</v>
       </c>
@@ -1342,8 +1573,20 @@
         <f t="shared" si="4"/>
         <v>6.2003586984370994E-3</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I18">
+        <f t="shared" si="5"/>
+        <v>0.19634703196347031</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="6"/>
+        <v>0.25114155251141551</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="7"/>
+        <v>0.55251141552511418</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>41</v>
       </c>
@@ -1365,8 +1608,20 @@
         <f t="shared" si="4"/>
         <v>6.2807495027739973E-3</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I19">
+        <f t="shared" si="5"/>
+        <v>0.18981481481481483</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="6"/>
+        <v>0.25462962962962965</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="7"/>
+        <v>0.55555555555555558</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>40</v>
       </c>
@@ -1388,8 +1643,20 @@
         <f t="shared" si="4"/>
         <v>6.1917946136420838E-3</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I20">
+        <f t="shared" si="5"/>
+        <v>0.18264840182648401</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="6"/>
+        <v>0.25570776255707761</v>
+      </c>
+      <c r="K20">
+        <f t="shared" si="7"/>
+        <v>0.56164383561643838</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>40</v>
       </c>
@@ -1411,8 +1678,20 @@
         <f t="shared" si="4"/>
         <v>6.3345044181837536E-3</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I21">
+        <f t="shared" si="5"/>
+        <v>0.18691588785046728</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="6"/>
+        <v>0.2570093457943925</v>
+      </c>
+      <c r="K21">
+        <f t="shared" si="7"/>
+        <v>0.55607476635514019</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>42</v>
       </c>
@@ -1434,8 +1713,20 @@
         <f t="shared" si="4"/>
         <v>6.1921088992375004E-3</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I22">
+        <f t="shared" si="5"/>
+        <v>0.19178082191780821</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="6"/>
+        <v>0.25570776255707761</v>
+      </c>
+      <c r="K22">
+        <f t="shared" si="7"/>
+        <v>0.55251141552511418</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>40</v>
       </c>
@@ -1457,8 +1748,20 @@
         <f t="shared" si="4"/>
         <v>6.3438359061112285E-3</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I23">
+        <f t="shared" si="5"/>
+        <v>0.18691588785046728</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="6"/>
+        <v>0.25233644859813081</v>
+      </c>
+      <c r="K23">
+        <f t="shared" si="7"/>
+        <v>0.56074766355140182</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>41</v>
       </c>
@@ -1480,8 +1783,20 @@
         <f t="shared" si="4"/>
         <v>6.1925790569006649E-3</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I24">
+        <f t="shared" si="5"/>
+        <v>0.18721461187214611</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="6"/>
+        <v>0.25570776255707761</v>
+      </c>
+      <c r="K24">
+        <f t="shared" si="7"/>
+        <v>0.55707762557077622</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>40</v>
       </c>
@@ -1503,8 +1818,20 @@
         <f t="shared" si="4"/>
         <v>6.3438359061112285E-3</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I25">
+        <f t="shared" si="5"/>
+        <v>0.18691588785046728</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="6"/>
+        <v>0.25233644859813081</v>
+      </c>
+      <c r="K25">
+        <f t="shared" si="7"/>
+        <v>0.56074766355140182</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>42</v>
       </c>
@@ -1526,8 +1853,20 @@
         <f t="shared" si="4"/>
         <v>6.2013927718192448E-3</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I26">
+        <f t="shared" si="5"/>
+        <v>0.19178082191780821</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="6"/>
+        <v>0.25114155251141551</v>
+      </c>
+      <c r="K26">
+        <f t="shared" si="7"/>
+        <v>0.55707762557077622</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>42</v>
       </c>
@@ -1549,8 +1888,20 @@
         <f t="shared" si="4"/>
         <v>6.1315776247675528E-3</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I27">
+        <f t="shared" si="5"/>
+        <v>0.19004524886877827</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="6"/>
+        <v>0.25791855203619912</v>
+      </c>
+      <c r="K27">
+        <f t="shared" si="7"/>
+        <v>0.55203619909502266</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>43</v>
       </c>
@@ -1572,8 +1923,20 @@
         <f t="shared" si="4"/>
         <v>6.1299964537210603E-3</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I28">
+        <f t="shared" si="5"/>
+        <v>0.19457013574660634</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="6"/>
+        <v>0.25791855203619912</v>
+      </c>
+      <c r="K28">
+        <f t="shared" si="7"/>
+        <v>0.54751131221719462</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>43</v>
       </c>
@@ -1595,8 +1958,20 @@
         <f t="shared" si="4"/>
         <v>6.1402184307212237E-3</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I29">
+        <f t="shared" si="5"/>
+        <v>0.19457013574660634</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="6"/>
+        <v>0.25339366515837103</v>
+      </c>
+      <c r="K29">
+        <f t="shared" si="7"/>
+        <v>0.55203619909502266</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>40</v>
       </c>
@@ -1618,8 +1993,20 @@
         <f t="shared" si="4"/>
         <v>6.2535240145573838E-3</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I30">
+        <f t="shared" si="5"/>
+        <v>0.18433179723502305</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="6"/>
+        <v>0.25345622119815669</v>
+      </c>
+      <c r="K30">
+        <f t="shared" si="7"/>
+        <v>0.56221198156682028</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>41</v>
       </c>
@@ -1641,8 +2028,20 @@
         <f t="shared" si="4"/>
         <v>6.2276671771311892E-3</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I31">
+        <f t="shared" si="5"/>
+        <v>0.18807339449541285</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="6"/>
+        <v>0.25229357798165136</v>
+      </c>
+      <c r="K31">
+        <f t="shared" si="7"/>
+        <v>0.55963302752293576</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>57</v>
       </c>
@@ -1664,8 +2063,20 @@
         <f t="shared" si="4"/>
         <v>4.4809156184203421E-3</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I32">
+        <f t="shared" si="5"/>
+        <v>0.18874172185430463</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="6"/>
+        <v>0.26158940397350994</v>
+      </c>
+      <c r="K32">
+        <f t="shared" si="7"/>
+        <v>0.54966887417218546</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>57</v>
       </c>
@@ -1687,8 +2098,20 @@
         <f t="shared" si="4"/>
         <v>4.4358778021281655E-3</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I33">
+        <f t="shared" si="5"/>
+        <v>0.18688524590163935</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="6"/>
+        <v>0.26229508196721313</v>
+      </c>
+      <c r="K33">
+        <f t="shared" si="7"/>
+        <v>0.55081967213114758</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>60</v>
       </c>
@@ -1710,8 +2133,20 @@
         <f t="shared" si="4"/>
         <v>4.388961892247043E-3</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I34">
+        <f t="shared" si="5"/>
+        <v>0.19480519480519481</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="6"/>
+        <v>0.26298701298701299</v>
+      </c>
+      <c r="K34">
+        <f t="shared" si="7"/>
+        <v>0.54220779220779225</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>58</v>
       </c>
@@ -1733,8 +2168,20 @@
         <f t="shared" si="4"/>
         <v>4.372687521022536E-3</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I35">
+        <f t="shared" si="5"/>
+        <v>0.18770226537216828</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="6"/>
+        <v>0.26537216828478966</v>
+      </c>
+      <c r="K35">
+        <f t="shared" si="7"/>
+        <v>0.54692556634304212</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>56</v>
       </c>
@@ -1756,8 +2203,20 @@
         <f t="shared" si="4"/>
         <v>4.4946254027563425E-3</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I36">
+        <f t="shared" si="5"/>
+        <v>0.18604651162790697</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="6"/>
+        <v>0.26245847176079734</v>
+      </c>
+      <c r="K36">
+        <f t="shared" si="7"/>
+        <v>0.55149501661129563</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>59</v>
       </c>
@@ -1779,8 +2238,20 @@
         <f t="shared" si="4"/>
         <v>4.3903203888569489E-3</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I37">
+        <f t="shared" si="5"/>
+        <v>0.19155844155844157</v>
+      </c>
+      <c r="J37">
+        <f t="shared" si="6"/>
+        <v>0.26298701298701299</v>
+      </c>
+      <c r="K37">
+        <f t="shared" si="7"/>
+        <v>0.54545454545454541</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>56</v>
       </c>
@@ -1802,8 +2273,20 @@
         <f t="shared" si="4"/>
         <v>4.4946254027563425E-3</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I38">
+        <f t="shared" si="5"/>
+        <v>0.18604651162790697</v>
+      </c>
+      <c r="J38">
+        <f t="shared" si="6"/>
+        <v>0.26245847176079734</v>
+      </c>
+      <c r="K38">
+        <f t="shared" si="7"/>
+        <v>0.55149501661129563</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>57</v>
       </c>
@@ -1825,8 +2308,20 @@
         <f t="shared" si="4"/>
         <v>4.4940759907394802E-3</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I39">
+        <f t="shared" si="5"/>
+        <v>0.18936877076411959</v>
+      </c>
+      <c r="J39">
+        <f t="shared" si="6"/>
+        <v>0.26245847176079734</v>
+      </c>
+      <c r="K39">
+        <f t="shared" si="7"/>
+        <v>0.54817275747508309</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>57</v>
       </c>
@@ -1848,8 +2343,20 @@
         <f t="shared" si="4"/>
         <v>4.4809156184203421E-3</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I40">
+        <f t="shared" si="5"/>
+        <v>0.18874172185430463</v>
+      </c>
+      <c r="J40">
+        <f t="shared" si="6"/>
+        <v>0.26158940397350994</v>
+      </c>
+      <c r="K40">
+        <f t="shared" si="7"/>
+        <v>0.54966887417218546</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>59</v>
       </c>
@@ -1871,8 +2378,20 @@
         <f t="shared" si="4"/>
         <v>4.4341159815156125E-3</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I41">
+        <f t="shared" si="5"/>
+        <v>0.19344262295081968</v>
+      </c>
+      <c r="J41">
+        <f t="shared" si="6"/>
+        <v>0.26229508196721313</v>
+      </c>
+      <c r="K41">
+        <f t="shared" si="7"/>
+        <v>0.54426229508196722</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>58</v>
       </c>
@@ -1894,8 +2413,20 @@
         <f t="shared" si="4"/>
         <v>4.4670487877075428E-3</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I42">
+        <f t="shared" si="5"/>
+        <v>0.19141914191419143</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="6"/>
+        <v>0.26072607260726072</v>
+      </c>
+      <c r="K42">
+        <f t="shared" si="7"/>
+        <v>0.54785478547854782</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>60</v>
       </c>
@@ -1917,8 +2448,20 @@
         <f t="shared" si="4"/>
         <v>4.2564775173847408E-3</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I43">
+        <f t="shared" si="5"/>
+        <v>0.1892744479495268</v>
+      </c>
+      <c r="J43">
+        <f t="shared" si="6"/>
+        <v>0.26813880126182965</v>
+      </c>
+      <c r="K43">
+        <f t="shared" si="7"/>
+        <v>0.54258675078864349</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>56</v>
       </c>
@@ -1940,8 +2483,20 @@
         <f t="shared" si="4"/>
         <v>4.5138133565368723E-3</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I44">
+        <f t="shared" si="5"/>
+        <v>0.18666666666666668</v>
+      </c>
+      <c r="J44">
+        <f t="shared" si="6"/>
+        <v>0.26</v>
+      </c>
+      <c r="K44">
+        <f t="shared" si="7"/>
+        <v>0.55333333333333334</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>56</v>
       </c>
@@ -1963,8 +2518,20 @@
         <f t="shared" si="4"/>
         <v>4.5079503852248513E-3</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I45">
+        <f t="shared" si="5"/>
+        <v>0.18666666666666668</v>
+      </c>
+      <c r="J45">
+        <f t="shared" si="6"/>
+        <v>0.26333333333333331</v>
+      </c>
+      <c r="K45">
+        <f t="shared" si="7"/>
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>60</v>
       </c>
@@ -1986,8 +2553,20 @@
         <f t="shared" si="4"/>
         <v>4.388961892247043E-3</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I46">
+        <f t="shared" si="5"/>
+        <v>0.19480519480519481</v>
+      </c>
+      <c r="J46">
+        <f t="shared" si="6"/>
+        <v>0.26298701298701299</v>
+      </c>
+      <c r="K46">
+        <f t="shared" si="7"/>
+        <v>0.54220779220779225</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>56</v>
       </c>
@@ -2009,8 +2588,20 @@
         <f t="shared" si="4"/>
         <v>4.5273700096035117E-3</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I47">
+        <f t="shared" si="5"/>
+        <v>0.18729096989966554</v>
+      </c>
+      <c r="J47">
+        <f t="shared" si="6"/>
+        <v>0.2608695652173913</v>
+      </c>
+      <c r="K47">
+        <f t="shared" si="7"/>
+        <v>0.55183946488294311</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>58</v>
       </c>
@@ -2032,8 +2623,20 @@
         <f t="shared" si="4"/>
         <v>4.4480171489817795E-3</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I48">
+        <f t="shared" si="5"/>
+        <v>0.19078947368421054</v>
+      </c>
+      <c r="J48">
+        <f t="shared" si="6"/>
+        <v>0.26315789473684209</v>
+      </c>
+      <c r="K48">
+        <f t="shared" si="7"/>
+        <v>0.54605263157894735</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>59</v>
       </c>
@@ -2055,8 +2658,20 @@
         <f t="shared" si="4"/>
         <v>4.3716984568945329E-3</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I49">
+        <f t="shared" si="5"/>
+        <v>0.19093851132686085</v>
+      </c>
+      <c r="J49">
+        <f t="shared" si="6"/>
+        <v>0.26537216828478966</v>
+      </c>
+      <c r="K49">
+        <f t="shared" si="7"/>
+        <v>0.5436893203883495</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>60</v>
       </c>
@@ -2078,8 +2693,20 @@
         <f t="shared" si="4"/>
         <v>4.3582027601950816E-3</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I50">
+        <f t="shared" si="5"/>
+        <v>0.19354838709677419</v>
+      </c>
+      <c r="J50">
+        <f t="shared" si="6"/>
+        <v>0.26451612903225807</v>
+      </c>
+      <c r="K50">
+        <f t="shared" si="7"/>
+        <v>0.54193548387096779</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>57</v>
       </c>
@@ -2101,8 +2728,20 @@
         <f t="shared" si="4"/>
         <v>4.4358778021281655E-3</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I51">
+        <f t="shared" si="5"/>
+        <v>0.18688524590163935</v>
+      </c>
+      <c r="J51">
+        <f t="shared" si="6"/>
+        <v>0.26229508196721313</v>
+      </c>
+      <c r="K51">
+        <f t="shared" si="7"/>
+        <v>0.55081967213114758</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>60</v>
       </c>
@@ -2124,8 +2763,20 @@
         <f t="shared" si="4"/>
         <v>4.3767096522078939E-3</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I52">
+        <f t="shared" si="5"/>
+        <v>0.1941747572815534</v>
+      </c>
+      <c r="J52">
+        <f t="shared" si="6"/>
+        <v>0.26213592233009708</v>
+      </c>
+      <c r="K52">
+        <f t="shared" si="7"/>
+        <v>0.5436893203883495</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>57</v>
       </c>
@@ -2147,8 +2798,20 @@
         <f t="shared" si="4"/>
         <v>4.4358778021281655E-3</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I53">
+        <f t="shared" si="5"/>
+        <v>0.18688524590163935</v>
+      </c>
+      <c r="J53">
+        <f t="shared" si="6"/>
+        <v>0.26229508196721313</v>
+      </c>
+      <c r="K53">
+        <f t="shared" si="7"/>
+        <v>0.55081967213114758</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>59</v>
       </c>
@@ -2170,8 +2833,20 @@
         <f t="shared" si="4"/>
         <v>4.3530082396227394E-3</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I54">
+        <f t="shared" si="5"/>
+        <v>0.19032258064516128</v>
+      </c>
+      <c r="J54">
+        <f t="shared" si="6"/>
+        <v>0.26774193548387099</v>
+      </c>
+      <c r="K54">
+        <f t="shared" si="7"/>
+        <v>0.54193548387096779</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>56</v>
       </c>
@@ -2193,8 +2868,20 @@
         <f t="shared" si="4"/>
         <v>4.4884524360055498E-3</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I55">
+        <f t="shared" si="5"/>
+        <v>0.18604651162790697</v>
+      </c>
+      <c r="J55">
+        <f t="shared" si="6"/>
+        <v>0.26578073089700999</v>
+      </c>
+      <c r="K55">
+        <f t="shared" si="7"/>
+        <v>0.54817275747508309</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>58</v>
       </c>
@@ -2216,8 +2903,20 @@
         <f t="shared" si="4"/>
         <v>4.3850490707872209E-3</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I56">
+        <f t="shared" si="5"/>
+        <v>0.18831168831168832</v>
+      </c>
+      <c r="J56">
+        <f t="shared" si="6"/>
+        <v>0.26623376623376621</v>
+      </c>
+      <c r="K56">
+        <f t="shared" si="7"/>
+        <v>0.54545454545454541</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>57</v>
       </c>
@@ -2239,8 +2938,20 @@
         <f t="shared" si="4"/>
         <v>4.4358778021281655E-3</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I57">
+        <f t="shared" si="5"/>
+        <v>0.18688524590163935</v>
+      </c>
+      <c r="J57">
+        <f t="shared" si="6"/>
+        <v>0.26229508196721313</v>
+      </c>
+      <c r="K57">
+        <f t="shared" si="7"/>
+        <v>0.55081967213114758</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>58</v>
       </c>
@@ -2262,8 +2973,20 @@
         <f t="shared" si="4"/>
         <v>4.4352375640719201E-3</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I58">
+        <f t="shared" si="5"/>
+        <v>0.1901639344262295</v>
+      </c>
+      <c r="J58">
+        <f t="shared" si="6"/>
+        <v>0.26229508196721313</v>
+      </c>
+      <c r="K58">
+        <f t="shared" si="7"/>
+        <v>0.54754098360655734</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>57</v>
       </c>
@@ -2285,8 +3008,20 @@
         <f t="shared" si="4"/>
         <v>4.4677492709810319E-3</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I59">
+        <f t="shared" si="5"/>
+        <v>0.18811881188118812</v>
+      </c>
+      <c r="J59">
+        <f t="shared" si="6"/>
+        <v>0.26072607260726072</v>
+      </c>
+      <c r="K59">
+        <f t="shared" si="7"/>
+        <v>0.55115511551155116</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>57</v>
       </c>
@@ -2308,8 +3043,20 @@
         <f t="shared" si="4"/>
         <v>4.4358778021281655E-3</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I60">
+        <f t="shared" si="5"/>
+        <v>0.18688524590163935</v>
+      </c>
+      <c r="J60">
+        <f t="shared" si="6"/>
+        <v>0.26229508196721313</v>
+      </c>
+      <c r="K60">
+        <f t="shared" si="7"/>
+        <v>0.55081967213114758</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>44</v>
       </c>
@@ -2331,8 +3078,20 @@
         <f t="shared" si="4"/>
         <v>5.7942592262435373E-3</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I61">
+        <f t="shared" si="5"/>
+        <v>0.18803418803418803</v>
+      </c>
+      <c r="J61">
+        <f t="shared" si="6"/>
+        <v>0.25641025641025639</v>
+      </c>
+      <c r="K61">
+        <f t="shared" si="7"/>
+        <v>0.55555555555555558</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>44</v>
       </c>
@@ -2354,8 +3113,20 @@
         <f t="shared" si="4"/>
         <v>5.7852722217239215E-3</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I62">
+        <f t="shared" si="5"/>
+        <v>0.18803418803418803</v>
+      </c>
+      <c r="J62">
+        <f t="shared" si="6"/>
+        <v>0.2606837606837607</v>
+      </c>
+      <c r="K62">
+        <f t="shared" si="7"/>
+        <v>0.55128205128205132</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>43</v>
       </c>
@@ -2377,8 +3148,20 @@
         <f t="shared" si="4"/>
         <v>5.8948144054527035E-3</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I63">
+        <f t="shared" si="5"/>
+        <v>0.18695652173913044</v>
+      </c>
+      <c r="J63">
+        <f t="shared" si="6"/>
+        <v>0.2565217391304348</v>
+      </c>
+      <c r="K63">
+        <f t="shared" si="7"/>
+        <v>0.55652173913043479</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>46</v>
       </c>
@@ -2400,8 +3183,20 @@
         <f t="shared" si="4"/>
         <v>5.7077120481394631E-3</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I64">
+        <f t="shared" si="5"/>
+        <v>0.1940928270042194</v>
+      </c>
+      <c r="J64">
+        <f t="shared" si="6"/>
+        <v>0.26160337552742619</v>
+      </c>
+      <c r="K64">
+        <f t="shared" si="7"/>
+        <v>0.54430379746835444</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>45</v>
       </c>
@@ -2423,8 +3218,20 @@
         <f t="shared" si="4"/>
         <v>5.8474189127455459E-3</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I65">
+        <f t="shared" si="5"/>
+        <v>0.19396551724137931</v>
+      </c>
+      <c r="J65">
+        <f t="shared" si="6"/>
+        <v>0.25431034482758619</v>
+      </c>
+      <c r="K65">
+        <f t="shared" si="7"/>
+        <v>0.55172413793103448</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>45</v>
       </c>
@@ -2446,8 +3253,20 @@
         <f t="shared" si="4"/>
         <v>5.762272747576719E-3</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I66">
+        <f t="shared" si="5"/>
+        <v>0.19148936170212766</v>
+      </c>
+      <c r="J66">
+        <f t="shared" si="6"/>
+        <v>0.25957446808510637</v>
+      </c>
+      <c r="K66">
+        <f t="shared" si="7"/>
+        <v>0.54893617021276597</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>44</v>
       </c>
@@ -2458,19 +3277,31 @@
         <v>127</v>
       </c>
       <c r="E67">
-        <f t="shared" ref="E67:E90" si="6">A67/($A67^2 + $B67^2 + $C67^2)</f>
+        <f t="shared" ref="E67:E90" si="10">A67/($A67^2 + $B67^2 + $C67^2)</f>
         <v>2.0421423930195859E-3</v>
       </c>
       <c r="F67">
-        <f t="shared" ref="F67:F90" si="7">B67/($A67^2 + $B67^2 + $C67^2)</f>
+        <f t="shared" ref="F67:F90" si="11">B67/($A67^2 + $B67^2 + $C67^2)</f>
         <v>2.7383272997308084E-3</v>
       </c>
       <c r="G67">
-        <f t="shared" ref="G67:G90" si="8">C67/($A67^2 + $B67^2 + $C67^2)</f>
+        <f t="shared" ref="G67:G90" si="12">C67/($A67^2 + $B67^2 + $C67^2)</f>
         <v>5.8943655434883502E-3</v>
       </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I67">
+        <f t="shared" ref="I67:I90" si="13">A67/($A67+$B67+$C67)</f>
+        <v>0.19130434782608696</v>
+      </c>
+      <c r="J67">
+        <f t="shared" ref="J67:J90" si="14">B67/($A67+$B67+$C67)</f>
+        <v>0.2565217391304348</v>
+      </c>
+      <c r="K67">
+        <f t="shared" ref="K67:K90" si="15">C67/($A67+$B67+$C67)</f>
+        <v>0.55217391304347829</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>44</v>
       </c>
@@ -2481,19 +3312,31 @@
         <v>127</v>
       </c>
       <c r="E68">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0421423930195859E-3</v>
       </c>
       <c r="F68">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7383272997308084E-3</v>
       </c>
       <c r="G68">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.8943655434883502E-3</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I68">
+        <f t="shared" si="13"/>
+        <v>0.19130434782608696</v>
+      </c>
+      <c r="J68">
+        <f t="shared" si="14"/>
+        <v>0.2565217391304348</v>
+      </c>
+      <c r="K68">
+        <f t="shared" si="15"/>
+        <v>0.55217391304347829</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>44</v>
       </c>
@@ -2504,19 +3347,31 @@
         <v>129</v>
       </c>
       <c r="E69">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>1.9840375163457636E-3</v>
       </c>
       <c r="F69">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7055057041078597E-3</v>
       </c>
       <c r="G69">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.8168372638318982E-3</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I69">
+        <f t="shared" si="13"/>
+        <v>0.18884120171673821</v>
+      </c>
+      <c r="J69">
+        <f t="shared" si="14"/>
+        <v>0.25751072961373389</v>
+      </c>
+      <c r="K69">
+        <f t="shared" si="15"/>
+        <v>0.55364806866952787</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>44</v>
       </c>
@@ -2527,19 +3382,31 @@
         <v>127</v>
       </c>
       <c r="E70">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0421423930195859E-3</v>
       </c>
       <c r="F70">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7383272997308084E-3</v>
       </c>
       <c r="G70">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.8943655434883502E-3</v>
       </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I70">
+        <f t="shared" si="13"/>
+        <v>0.19130434782608696</v>
+      </c>
+      <c r="J70">
+        <f t="shared" si="14"/>
+        <v>0.2565217391304348</v>
+      </c>
+      <c r="K70">
+        <f t="shared" si="15"/>
+        <v>0.55217391304347829</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>40</v>
       </c>
@@ -2550,19 +3417,31 @@
         <v>128</v>
       </c>
       <c r="E71">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>1.8634987188446308E-3</v>
       </c>
       <c r="F71">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7486606102958304E-3</v>
       </c>
       <c r="G71">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.9631959003028185E-3</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I71">
+        <f t="shared" si="13"/>
+        <v>0.1762114537444934</v>
+      </c>
+      <c r="J71">
+        <f t="shared" si="14"/>
+        <v>0.25991189427312777</v>
+      </c>
+      <c r="K71">
+        <f t="shared" si="15"/>
+        <v>0.56387665198237891</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>45</v>
       </c>
@@ -2573,19 +3452,31 @@
         <v>126</v>
       </c>
       <c r="E72">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.1045739406977833E-3</v>
       </c>
       <c r="F72">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.75933027780376E-3</v>
       </c>
       <c r="G72">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.8928070339537928E-3</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I72">
+        <f t="shared" si="13"/>
+        <v>0.19565217391304349</v>
+      </c>
+      <c r="J72">
+        <f t="shared" si="14"/>
+        <v>0.2565217391304348</v>
+      </c>
+      <c r="K72">
+        <f t="shared" si="15"/>
+        <v>0.54782608695652169</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>43</v>
       </c>
@@ -2596,19 +3487,31 @@
         <v>129</v>
       </c>
       <c r="E73">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>1.9571253015338401E-3</v>
       </c>
       <c r="F73">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.6853579718720132E-3</v>
       </c>
       <c r="G73">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.8713759046015203E-3</v>
       </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I73">
+        <f t="shared" si="13"/>
+        <v>0.18614718614718614</v>
+      </c>
+      <c r="J73">
+        <f t="shared" si="14"/>
+        <v>0.25541125541125542</v>
+      </c>
+      <c r="K73">
+        <f t="shared" si="15"/>
+        <v>0.55844155844155841</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>45</v>
       </c>
@@ -2619,19 +3522,31 @@
         <v>129</v>
       </c>
       <c r="E74">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0100951445035063E-3</v>
       </c>
       <c r="F74">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7247956403269754E-3</v>
       </c>
       <c r="G74">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.762272747576719E-3</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I74">
+        <f t="shared" si="13"/>
+        <v>0.19148936170212766</v>
+      </c>
+      <c r="J74">
+        <f t="shared" si="14"/>
+        <v>0.25957446808510637</v>
+      </c>
+      <c r="K74">
+        <f t="shared" si="15"/>
+        <v>0.54893617021276597</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>42</v>
       </c>
@@ -2642,19 +3557,31 @@
         <v>127</v>
       </c>
       <c r="E75">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>1.9865670229874182E-3</v>
       </c>
       <c r="F75">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.6960552454829249E-3</v>
       </c>
       <c r="G75">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>6.0070002837952887E-3</v>
       </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I75">
+        <f t="shared" si="13"/>
+        <v>0.18584070796460178</v>
+      </c>
+      <c r="J75">
+        <f t="shared" si="14"/>
+        <v>0.25221238938053098</v>
+      </c>
+      <c r="K75">
+        <f t="shared" si="15"/>
+        <v>0.56194690265486724</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>42</v>
       </c>
@@ -2665,19 +3592,31 @@
         <v>126</v>
       </c>
       <c r="E76">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>1.999619120167587E-3</v>
       </c>
       <c r="F76">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7613787849933348E-3</v>
       </c>
       <c r="G76">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.9988573605027611E-3</v>
       </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I76">
+        <f t="shared" si="13"/>
+        <v>0.18584070796460178</v>
+      </c>
+      <c r="J76">
+        <f t="shared" si="14"/>
+        <v>0.25663716814159293</v>
+      </c>
+      <c r="K76">
+        <f t="shared" si="15"/>
+        <v>0.55752212389380529</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>42</v>
       </c>
@@ -2688,19 +3627,31 @@
         <v>127</v>
       </c>
       <c r="E77">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>1.9865670229874182E-3</v>
       </c>
       <c r="F77">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.6960552454829249E-3</v>
       </c>
       <c r="G77">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>6.0070002837952887E-3</v>
       </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I77">
+        <f t="shared" si="13"/>
+        <v>0.18584070796460178</v>
+      </c>
+      <c r="J77">
+        <f t="shared" si="14"/>
+        <v>0.25221238938053098</v>
+      </c>
+      <c r="K77">
+        <f t="shared" si="15"/>
+        <v>0.56194690265486724</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>46</v>
       </c>
@@ -2711,19 +3662,31 @@
         <v>129</v>
       </c>
       <c r="E78">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0464454132929975E-3</v>
       </c>
       <c r="F78">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.713764569801584E-3</v>
       </c>
       <c r="G78">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.738944745973841E-3</v>
       </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I78">
+        <f t="shared" si="13"/>
+        <v>0.19491525423728814</v>
+      </c>
+      <c r="J78">
+        <f t="shared" si="14"/>
+        <v>0.25847457627118642</v>
+      </c>
+      <c r="K78">
+        <f t="shared" si="15"/>
+        <v>0.54661016949152541</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>43</v>
       </c>
@@ -2734,19 +3697,31 @@
         <v>128</v>
       </c>
       <c r="E79">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>1.9694957174918701E-3</v>
       </c>
       <c r="F79">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7481335592909814E-3</v>
       </c>
       <c r="G79">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.8626849264874275E-3</v>
       </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I79">
+        <f t="shared" si="13"/>
+        <v>0.18614718614718614</v>
+      </c>
+      <c r="J79">
+        <f t="shared" si="14"/>
+        <v>0.25974025974025972</v>
+      </c>
+      <c r="K79">
+        <f t="shared" si="15"/>
+        <v>0.55411255411255411</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>44</v>
       </c>
@@ -2757,19 +3732,31 @@
         <v>127</v>
       </c>
       <c r="E80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0532922674879836E-3</v>
       </c>
       <c r="F80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7066125344159782E-3</v>
       </c>
       <c r="G80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.9265481357039526E-3</v>
       </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I80">
+        <f t="shared" si="13"/>
+        <v>0.19213973799126638</v>
+      </c>
+      <c r="J80">
+        <f t="shared" si="14"/>
+        <v>0.25327510917030566</v>
+      </c>
+      <c r="K80">
+        <f t="shared" si="15"/>
+        <v>0.55458515283842791</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>42</v>
       </c>
@@ -2780,19 +3767,31 @@
         <v>128</v>
       </c>
       <c r="E81">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>1.9628919942047949E-3</v>
       </c>
       <c r="F81">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.663924849277936E-3</v>
       </c>
       <c r="G81">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.9821470299574707E-3</v>
       </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I81">
+        <f t="shared" si="13"/>
+        <v>0.18502202643171806</v>
+      </c>
+      <c r="J81">
+        <f t="shared" si="14"/>
+        <v>0.25110132158590309</v>
+      </c>
+      <c r="K81">
+        <f t="shared" si="15"/>
+        <v>0.56387665198237891</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>43</v>
       </c>
@@ -2803,19 +3802,31 @@
         <v>127</v>
       </c>
       <c r="E82">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0257219578838272E-3</v>
       </c>
       <c r="F82">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.6852593395204219E-3</v>
       </c>
       <c r="G82">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.9829462477033963E-3</v>
       </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I82">
+        <f t="shared" si="13"/>
+        <v>0.1894273127753304</v>
+      </c>
+      <c r="J82">
+        <f t="shared" si="14"/>
+        <v>0.25110132158590309</v>
+      </c>
+      <c r="K82">
+        <f t="shared" si="15"/>
+        <v>0.55947136563876654</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>43</v>
       </c>
@@ -2826,19 +3837,31 @@
         <v>128</v>
       </c>
       <c r="E83">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>1.9802892143317677E-3</v>
       </c>
       <c r="F83">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7171410150133553E-3</v>
       </c>
       <c r="G83">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.8948144054527035E-3</v>
       </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I83">
+        <f t="shared" si="13"/>
+        <v>0.18695652173913044</v>
+      </c>
+      <c r="J83">
+        <f t="shared" si="14"/>
+        <v>0.2565217391304348</v>
+      </c>
+      <c r="K83">
+        <f t="shared" si="15"/>
+        <v>0.55652173913043479</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>44</v>
       </c>
@@ -2849,19 +3872,31 @@
         <v>128</v>
       </c>
       <c r="E84">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0182560433007661E-3</v>
       </c>
       <c r="F84">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.706297876244209E-3</v>
       </c>
       <c r="G84">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.8712903077840469E-3</v>
       </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I84">
+        <f t="shared" si="13"/>
+        <v>0.19047619047619047</v>
+      </c>
+      <c r="J84">
+        <f t="shared" si="14"/>
+        <v>0.25541125541125542</v>
+      </c>
+      <c r="K84">
+        <f t="shared" si="15"/>
+        <v>0.55411255411255411</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>44</v>
       </c>
@@ -2872,19 +3907,31 @@
         <v>126</v>
       </c>
       <c r="E85">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0778239516433699E-3</v>
       </c>
       <c r="F85">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7389497544389875E-3</v>
       </c>
       <c r="G85">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.9501322251605589E-3</v>
       </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I85">
+        <f t="shared" si="13"/>
+        <v>0.19298245614035087</v>
+      </c>
+      <c r="J85">
+        <f t="shared" si="14"/>
+        <v>0.25438596491228072</v>
+      </c>
+      <c r="K85">
+        <f t="shared" si="15"/>
+        <v>0.55263157894736847</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>46</v>
       </c>
@@ -2895,19 +3942,31 @@
         <v>129</v>
       </c>
       <c r="E86">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0353081722047695E-3</v>
       </c>
       <c r="F86">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7432414494933852E-3</v>
       </c>
       <c r="G86">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.7077120481394631E-3</v>
       </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I86">
+        <f t="shared" si="13"/>
+        <v>0.1940928270042194</v>
+      </c>
+      <c r="J86">
+        <f t="shared" si="14"/>
+        <v>0.26160337552742619</v>
+      </c>
+      <c r="K86">
+        <f t="shared" si="15"/>
+        <v>0.54430379746835444</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>44</v>
       </c>
@@ -2918,19 +3977,31 @@
         <v>128</v>
       </c>
       <c r="E87">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0072992700729928E-3</v>
       </c>
       <c r="F87">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7372262773722629E-3</v>
       </c>
       <c r="G87">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.8394160583941602E-3</v>
       </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I87">
+        <f t="shared" si="13"/>
+        <v>0.18965517241379309</v>
+      </c>
+      <c r="J87">
+        <f t="shared" si="14"/>
+        <v>0.25862068965517243</v>
+      </c>
+      <c r="K87">
+        <f t="shared" si="15"/>
+        <v>0.55172413793103448</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>42</v>
       </c>
@@ -2941,19 +4012,31 @@
         <v>127</v>
       </c>
       <c r="E88">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>1.9865670229874182E-3</v>
       </c>
       <c r="F88">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.6960552454829249E-3</v>
       </c>
       <c r="G88">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>6.0070002837952887E-3</v>
       </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I88">
+        <f t="shared" si="13"/>
+        <v>0.18584070796460178</v>
+      </c>
+      <c r="J88">
+        <f t="shared" si="14"/>
+        <v>0.25221238938053098</v>
+      </c>
+      <c r="K88">
+        <f t="shared" si="15"/>
+        <v>0.56194690265486724</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>45</v>
       </c>
@@ -2964,19 +4047,31 @@
         <v>129</v>
       </c>
       <c r="E89">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0100951445035063E-3</v>
       </c>
       <c r="F89">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.7247956403269754E-3</v>
       </c>
       <c r="G89">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.762272747576719E-3</v>
       </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I89">
+        <f t="shared" si="13"/>
+        <v>0.19148936170212766</v>
+      </c>
+      <c r="J89">
+        <f t="shared" si="14"/>
+        <v>0.25957446808510637</v>
+      </c>
+      <c r="K89">
+        <f t="shared" si="15"/>
+        <v>0.54893617021276597</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>44</v>
       </c>
@@ -2987,16 +4082,28 @@
         <v>128</v>
       </c>
       <c r="E90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>2.0182560433007661E-3</v>
       </c>
       <c r="F90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>2.706297876244209E-3</v>
       </c>
       <c r="G90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>5.8712903077840469E-3</v>
+      </c>
+      <c r="I90">
+        <f t="shared" si="13"/>
+        <v>0.19047619047619047</v>
+      </c>
+      <c r="J90">
+        <f t="shared" si="14"/>
+        <v>0.25541125541125542</v>
+      </c>
+      <c r="K90">
+        <f t="shared" si="15"/>
+        <v>0.55411255411255411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>